<commit_message>
securizado y mando sin desocupar
</commit_message>
<xml_diff>
--- a/app/uploads/Prueba asignar camas.xlsx
+++ b/app/uploads/Prueba asignar camas.xlsx
@@ -25,9 +25,6 @@
     <t>genero</t>
   </si>
   <si>
-    <t>Pepito</t>
-  </si>
-  <si>
     <t>Joaquín</t>
   </si>
   <si>
@@ -71,6 +68,9 @@
   </si>
   <si>
     <t>ham</t>
+  </si>
+  <si>
+    <t>Pepe</t>
   </si>
 </sst>
 </file>
@@ -426,16 +426,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>11</v>
-      </c>
-      <c r="E1" t="s">
-        <v>12</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
@@ -446,48 +446,48 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2">
         <v>400</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
       </c>
       <c r="D3">
         <v>401</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
securizado cerrado de pestaña y ventana y scroll corregido
</commit_message>
<xml_diff>
--- a/app/uploads/Prueba asignar camas.xlsx
+++ b/app/uploads/Prueba asignar camas.xlsx
@@ -25,9 +25,6 @@
     <t>genero</t>
   </si>
   <si>
-    <t>Joaquín</t>
-  </si>
-  <si>
     <t>407A</t>
   </si>
   <si>
@@ -37,9 +34,6 @@
     <t>M</t>
   </si>
   <si>
-    <t>F</t>
-  </si>
-  <si>
     <t>apellido1</t>
   </si>
   <si>
@@ -71,6 +65,12 @@
   </si>
   <si>
     <t>Pepe</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Mary</t>
   </si>
 </sst>
 </file>
@@ -426,16 +426,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>9</v>
-      </c>
-      <c r="D1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" t="s">
-        <v>11</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
@@ -446,48 +446,48 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>400</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>401</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" t="s">
         <v>5</v>
-      </c>
-      <c r="G3" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>